<commit_message>
Normalize two uppercase attendee names in departure workbook
</commit_message>
<xml_diff>
--- a/gs/departures.xlsx
+++ b/gs/departures.xlsx
@@ -141,7 +141,7 @@
     <t>3:25 PM - 7:50  PM</t>
   </si>
   <si>
-    <t>GUSTAVO MENENDEZ</t>
+    <t>Gustavo Menendez</t>
   </si>
   <si>
     <t>Oct 8</t>
@@ -222,7 +222,7 @@
     <t xml:space="preserve">German Rodriguez </t>
   </si>
   <si>
-    <t>EDUARDO ARTAVIA</t>
+    <t>Eduardo Artavia</t>
   </si>
   <si>
     <t>Abdiel Hernandez</t>

</xml_diff>